<commit_message>
Update Banxico_Minutes_Analysis.xlsx - 2026-10-10
</commit_message>
<xml_diff>
--- a/Banxico_Minutes_Analysis.xlsx
+++ b/Banxico_Minutes_Analysis.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L127"/>
+  <dimension ref="A1:L128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8050,6 +8050,66 @@
       <c r="L127" t="inlineStr">
         <is>
           <t>The decision to hold rates suggests a cautious approach, likely keeping the yield curve stable in the short term, but with potential upward pressure if inflation risks materialize.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>The policy decision was to hold the interest rate steady.</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>0</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>{"hold": 5}</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>The committee noted a slight moderation in global economic growth in Q3 2026, with advanced economies slowing while emerging markets maintained their pace. In Mexico, economic activity showed signs of stabilization with a notable GDP growth in Q2 2026.</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Headline inflation in advanced economies has risen due to energy prices, while core inflation remains persistent. In Mexico, inflation is expected to face upward pressures from global energy prices and geopolitical tensions.</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>The labor market in the US remains strong, supported by resilient internal demand and robust capital investment. In Mexico, the labor market is stabilizing with signs of recovery in industrial activity.</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>There was a consensus to hold rates, with no dissenting votes. The discussion focused on external risks and inflation pressures.</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>The committee remains cautious, emphasizing the need to monitor geopolitical developments and their impact on inflation and growth. Future policy moves will be data-dependent.</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>The decision to hold rates suggests a cautious approach, likely leading to stable yield curves and limited FX volatility unless geopolitical risks escalate.</t>
         </is>
       </c>
     </row>
@@ -8064,7 +8124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D127"/>
+  <dimension ref="A1:D128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10606,6 +10666,26 @@
       <c r="D127" t="inlineStr">
         <is>
           <t>Hold the policy rate steady.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>0</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>The policy decision was to hold the interest rate steady.</t>
         </is>
       </c>
     </row>
@@ -10620,7 +10700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C548"/>
+  <dimension ref="A1:C552"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19936,6 +20016,74 @@
       <c r="C548" t="inlineStr">
         <is>
           <t>The Mexican economy rebounded in Q2 2026, reducing immediate concerns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>hawkish</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Persistent inflation pressures in advanced economies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>hawkish</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Federal Reserve's rate hike and expectations of further increases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>dovish</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Moderation in global economic growth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>dovish</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Stabilization signs in Mexico's economic activity.</t>
         </is>
       </c>
     </row>

</xml_diff>